<commit_message>
Update bug report with evidence links
</commit_message>
<xml_diff>
--- a/Bug-Report.xlsx
+++ b/Bug-Report.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0. Documentos\Github\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0. Documentos\Github\qa-repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9087915-CA5F-4D82-836F-B367887C40F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F73459F-9D22-474C-907C-56694CC34521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1204,11 +1204,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D6" r:id="rId1" display="BUG-009_overview-direct-url-with-empty-cart.mp4" xr:uid="{DD5DAC95-F8D5-4373-A9BE-73474C742E85}"/>
-    <hyperlink ref="D5" r:id="rId2" display="BUG-008_overview-direct-url-skips-form.mp4" xr:uid="{ED1AF2FD-16DD-4A45-9949-F6FF57780CD6}"/>
-    <hyperlink ref="D4" r:id="rId3" display="BUG-007_checkout-with-only-spaces.mp4" xr:uid="{D2471659-5B00-4D8E-A03C-0B9F7A938487}"/>
-    <hyperlink ref="D3" r:id="rId4" display="BUG-006_checkout-with-invalid-characters.mp4" xr:uid="{2E56F9CE-5FD3-4A02-9D67-95BD03C43D6F}"/>
-    <hyperlink ref="D2" r:id="rId5" display="BUG-005_checkout-with-empty-cart.mp4" xr:uid="{02812482-AFD3-4D39-B8B9-102029BB4BD0}"/>
+    <hyperlink ref="D6" r:id="rId1" xr:uid="{DD5DAC95-F8D5-4373-A9BE-73474C742E85}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{ED1AF2FD-16DD-4A45-9949-F6FF57780CD6}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{D2471659-5B00-4D8E-A03C-0B9F7A938487}"/>
+    <hyperlink ref="D3" r:id="rId4" xr:uid="{2E56F9CE-5FD3-4A02-9D67-95BD03C43D6F}"/>
+    <hyperlink ref="D2" r:id="rId5" xr:uid="{02812482-AFD3-4D39-B8B9-102029BB4BD0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>